<commit_message>
data: update IDC to 202609 BCB release (Jul-2026)
IDC reaches 0.963 (vs 0.950 in Jun-2026); higher delinquency offsets improved credit composition.
</commit_message>
<xml_diff>
--- a/data/processed/idc_data.xlsx
+++ b/data/processed/idc_data.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componentes Brutos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IDC e Normalizados'!$A$1:$E$185</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Componentes Brutos'!$A$1:$D$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IDC e Normalizados'!$A$1:$E$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Componentes Brutos'!$A$1:$D$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3556,10 +3556,10 @@
         <v>0.903225806451613</v>
       </c>
       <c r="D178" s="2" t="n">
-        <v>0.9922483704090016</v>
+        <v>0.9892219518293673</v>
       </c>
       <c r="E178" s="2" t="n">
-        <v>0.9610930183031318</v>
+        <v>0.9600842121099203</v>
       </c>
     </row>
     <row r="179">
@@ -3575,10 +3575,10 @@
         <v>0.9677419354838708</v>
       </c>
       <c r="D179" s="2" t="n">
-        <v>0.920472930072725</v>
+        <v>0.9199343400923999</v>
       </c>
       <c r="E179" s="2" t="n">
-        <v>0.9627382885188652</v>
+        <v>0.9625587585254235</v>
       </c>
     </row>
     <row r="180">
@@ -3594,10 +3594,10 @@
         <v>1</v>
       </c>
       <c r="D180" s="2" t="n">
-        <v>0.9877814324465222</v>
+        <v>0.9872659511807742</v>
       </c>
       <c r="E180" s="2" t="n">
-        <v>0.9959271441488408</v>
+        <v>0.995755317060258</v>
       </c>
     </row>
     <row r="181">
@@ -3632,10 +3632,10 @@
         <v>0.9393939393939393</v>
       </c>
       <c r="D182" s="2" t="n">
-        <v>0.9534840917507833</v>
+        <v>0.9536895362579288</v>
       </c>
       <c r="E182" s="2" t="n">
-        <v>0.9603711084207899</v>
+        <v>0.9604395899231717</v>
       </c>
     </row>
     <row r="183">
@@ -3651,10 +3651,10 @@
         <v>1</v>
       </c>
       <c r="D183" s="2" t="n">
-        <v>0.9712941575502504</v>
+        <v>0.9714984708437086</v>
       </c>
       <c r="E183" s="2" t="n">
-        <v>0.9904313858500835</v>
+        <v>0.9904994902812362</v>
       </c>
     </row>
     <row r="184">
@@ -3670,10 +3670,10 @@
         <v>1</v>
       </c>
       <c r="D184" s="2" t="n">
-        <v>0.9496989605019228</v>
+        <v>0.9496890561364562</v>
       </c>
       <c r="E184" s="2" t="n">
-        <v>0.9832329868339743</v>
+        <v>0.9832296853788187</v>
       </c>
     </row>
     <row r="185">
@@ -3686,17 +3686,36 @@
         <v>1</v>
       </c>
       <c r="C185" s="2" t="n">
-        <v>0.9705882352941178</v>
+        <v>0.9428571428571431</v>
       </c>
       <c r="D185" s="2" t="n">
         <v>0.9070197678750417</v>
       </c>
       <c r="E185" s="2" t="n">
-        <v>0.9592026677230532</v>
+        <v>0.9499589702440616</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" s="2" t="n">
+        <v>0.8876718413864001</v>
+      </c>
+      <c r="E186" s="2" t="n">
+        <v>0.9625572804621334</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E185"/>
+  <autoFilter ref="A1:E186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3707,7 +3726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D185"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6567,7 +6586,7 @@
         <v>6.9</v>
       </c>
       <c r="D178" s="2" t="n">
-        <v>0.2476337155964247</v>
+        <v>0.2474370301084636</v>
       </c>
     </row>
     <row r="179">
@@ -6583,7 +6602,7 @@
         <v>7.1</v>
       </c>
       <c r="D179" s="2" t="n">
-        <v>0.2429690642487354</v>
+        <v>0.2429340615449442</v>
       </c>
     </row>
     <row r="180">
@@ -6599,7 +6618,7 @@
         <v>7.2</v>
       </c>
       <c r="D180" s="2" t="n">
-        <v>0.2473434114465776</v>
+        <v>0.2473099105670328</v>
       </c>
     </row>
     <row r="181">
@@ -6631,7 +6650,7 @@
         <v>7.2</v>
       </c>
       <c r="D182" s="2" t="n">
-        <v>0.2482663364677345</v>
+        <v>0.2482803673368081</v>
       </c>
     </row>
     <row r="183">
@@ -6647,7 +6666,7 @@
         <v>7.4</v>
       </c>
       <c r="D183" s="2" t="n">
-        <v>0.2494826780720774</v>
+        <v>0.2494966316847115</v>
       </c>
     </row>
     <row r="184">
@@ -6660,10 +6679,10 @@
         <v>28.5</v>
       </c>
       <c r="C184" s="3" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="D184" s="2" t="n">
-        <v>0.2480078302573855</v>
+        <v>0.2480071538369883</v>
       </c>
     </row>
     <row r="185">
@@ -6673,7 +6692,7 @@
         </is>
       </c>
       <c r="B185" s="3" t="n">
-        <v>28.9</v>
+        <v>28.7</v>
       </c>
       <c r="C185" s="3" t="n">
         <v>7.4</v>
@@ -6682,8 +6701,24 @@
         <v>0.2450930472230976</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="C186" s="3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D186" s="2" t="n">
+        <v>0.2437716771500794</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D185"/>
+  <autoFilter ref="A1:D186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>